<commit_message>
Mise à jour base joueurs [via Soccer FFL]
</commit_message>
<xml_diff>
--- a/database_joueurs_v2.xlsx
+++ b/database_joueurs_v2.xlsx
@@ -966,7 +966,11 @@
       <c r="E25" t="n">
         <v>7</v>
       </c>
-      <c r="F25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Surfeur</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">

</xml_diff>